<commit_message>
Add a proprietary Institution_ID to the sample reports (#289)
</commit_message>
<xml_diff>
--- a/source/_static/report/DRD1_sample_r51.xlsx
+++ b/source/_static/report/DRD1_sample_r51.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\office\counter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\siq\github\cop5\source\_static\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DEAD813-47EF-4B2A-B6FC-5C70137EC309}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1ED4A2-97E7-49B1-9284-8FD23E2F3B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DRD1_sample_r51" sheetId="1" r:id="rId1"/>
@@ -57,9 +57,6 @@
     <t>Institution_ID</t>
   </si>
   <si>
-    <t>ISNI:1234123412341234</t>
-  </si>
-  <si>
     <t>Metric_Types</t>
   </si>
   <si>
@@ -202,6 +199,9 @@
   </si>
   <si>
     <t>P1:DB3</t>
+  </si>
+  <si>
+    <t>P1:1234; ISNI:1234123412341234</t>
   </si>
 </sst>
 </file>
@@ -240,12 +240,12 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -371,7 +371,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" style="1" customWidth="1"/>
@@ -430,144 +430,144 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="L15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="M15" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M15" s="1" t="s">
+      <c r="N15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N15" s="1" t="s">
+      <c r="O15" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O15" s="1" t="s">
+      <c r="P15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="P15" s="1" t="s">
+      <c r="Q15" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="Q15" s="1" t="s">
+      <c r="R15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="R15" s="1" t="s">
+      <c r="S15" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="G16" s="2">
         <v>192008</v>
@@ -611,22 +611,22 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F17" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G17" s="2">
         <v>199413</v>
@@ -670,22 +670,22 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F18" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G18" s="2">
         <v>185698</v>
@@ -729,22 +729,22 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G19" s="2">
         <v>213928</v>
@@ -788,22 +788,22 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F20" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G20" s="2">
         <v>128358</v>
@@ -847,22 +847,22 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F21" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G21" s="2">
         <v>160460</v>
@@ -906,22 +906,22 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F22" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G22" s="2">
         <v>96396</v>
@@ -965,22 +965,22 @@
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F23" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G23" s="2">
         <v>195502</v>
@@ -1024,22 +1024,22 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F24" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G24" s="2">
         <v>187475</v>
@@ -1083,22 +1083,22 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F25" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G25" s="2">
         <v>197245</v>
@@ -1142,22 +1142,22 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F26" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G26" s="2">
         <v>72179</v>
@@ -1201,22 +1201,22 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F27" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G27" s="2">
         <v>54144</v>
@@ -1260,22 +1260,22 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F28" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G28" s="2">
         <v>194034</v>
@@ -1319,22 +1319,22 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F29" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G29" s="2">
         <v>203905</v>
@@ -1378,22 +1378,22 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F30" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G30" s="2">
         <v>189376</v>
@@ -1437,22 +1437,22 @@
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F31" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G31" s="2">
         <v>16981</v>
@@ -1496,22 +1496,22 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G32" s="2">
         <v>10189</v>
@@ -1555,22 +1555,22 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F33" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G33" s="2">
         <v>12739</v>
@@ -1614,22 +1614,22 @@
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F34" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G34" s="2">
         <v>7642</v>

</xml_diff>

<commit_message>
Add a proprietary Institution_ID to the sample reports (#326)
</commit_message>
<xml_diff>
--- a/source/_static/report/DRD1_sample_r51.xlsx
+++ b/source/_static/report/DRD1_sample_r51.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\office\counter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\siq\github\cop5\source\_static\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DEAD813-47EF-4B2A-B6FC-5C70137EC309}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1ED4A2-97E7-49B1-9284-8FD23E2F3B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DRD1_sample_r51" sheetId="1" r:id="rId1"/>
@@ -57,9 +57,6 @@
     <t>Institution_ID</t>
   </si>
   <si>
-    <t>ISNI:1234123412341234</t>
-  </si>
-  <si>
     <t>Metric_Types</t>
   </si>
   <si>
@@ -202,6 +199,9 @@
   </si>
   <si>
     <t>P1:DB3</t>
+  </si>
+  <si>
+    <t>P1:1234; ISNI:1234123412341234</t>
   </si>
 </sst>
 </file>
@@ -240,12 +240,12 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -371,7 +371,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" style="1" customWidth="1"/>
@@ -430,144 +430,144 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="L15" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="M15" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M15" s="1" t="s">
+      <c r="N15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N15" s="1" t="s">
+      <c r="O15" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O15" s="1" t="s">
+      <c r="P15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="P15" s="1" t="s">
+      <c r="Q15" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="Q15" s="1" t="s">
+      <c r="R15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="R15" s="1" t="s">
+      <c r="S15" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="G16" s="2">
         <v>192008</v>
@@ -611,22 +611,22 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D17" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F17" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G17" s="2">
         <v>199413</v>
@@ -670,22 +670,22 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F18" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G18" s="2">
         <v>185698</v>
@@ -729,22 +729,22 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F19" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G19" s="2">
         <v>213928</v>
@@ -788,22 +788,22 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F20" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G20" s="2">
         <v>128358</v>
@@ -847,22 +847,22 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F21" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G21" s="2">
         <v>160460</v>
@@ -906,22 +906,22 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>46</v>
-      </c>
       <c r="F22" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G22" s="2">
         <v>96396</v>
@@ -965,22 +965,22 @@
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F23" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G23" s="2">
         <v>195502</v>
@@ -1024,22 +1024,22 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F24" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G24" s="2">
         <v>187475</v>
@@ -1083,22 +1083,22 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F25" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G25" s="2">
         <v>197245</v>
@@ -1142,22 +1142,22 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F26" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G26" s="2">
         <v>72179</v>
@@ -1201,22 +1201,22 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F27" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G27" s="2">
         <v>54144</v>
@@ -1260,22 +1260,22 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F28" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G28" s="2">
         <v>194034</v>
@@ -1319,22 +1319,22 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F29" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G29" s="2">
         <v>203905</v>
@@ -1378,22 +1378,22 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F30" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G30" s="2">
         <v>189376</v>
@@ -1437,22 +1437,22 @@
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F31" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G31" s="2">
         <v>16981</v>
@@ -1496,22 +1496,22 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F32" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G32" s="2">
         <v>10189</v>
@@ -1555,22 +1555,22 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F33" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G33" s="2">
         <v>12739</v>
@@ -1614,22 +1614,22 @@
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="F34" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G34" s="2">
         <v>7642</v>

</xml_diff>